<commit_message>
Add dataset refresh commands
</commit_message>
<xml_diff>
--- a/data/generated/dher_de.xlsx
+++ b/data/generated/dher_de.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -126,6 +126,23 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Codex</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Refreshed from Yahoo Finance DHER.DE monthly history on 2026-03-11 01:30:59.
+https://finance.yahoo.com/quote/DHER.DE/history/
+Earliest reliable live month for this series: 2010-06-01.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -417,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +470,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B2" t="n">
@@ -473,7 +490,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B3" t="n">
@@ -493,7 +510,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B4" t="n">
@@ -513,7 +530,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="B5" t="n">
@@ -533,7 +550,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>45962</v>
       </c>
       <c r="B6" t="n">
@@ -553,7 +570,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="B7" t="n">
@@ -573,7 +590,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="B8" t="n">
@@ -593,7 +610,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>45870</v>
       </c>
       <c r="B9" t="n">
@@ -613,7 +630,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="B10" t="n">
@@ -633,7 +650,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>45809</v>
       </c>
       <c r="B11" t="n">
@@ -653,7 +670,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="B12" t="n">
@@ -673,7 +690,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="B13" t="n">
@@ -693,7 +710,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>45717</v>
       </c>
       <c r="B14" t="n">
@@ -713,7 +730,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>45689</v>
       </c>
       <c r="B15" t="n">
@@ -733,7 +750,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>45658</v>
       </c>
       <c r="B16" t="n">
@@ -753,7 +770,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>45627</v>
       </c>
       <c r="B17" t="n">
@@ -773,7 +790,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>45597</v>
       </c>
       <c r="B18" t="n">
@@ -793,7 +810,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="B19" t="n">
@@ -813,7 +830,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>45536</v>
       </c>
       <c r="B20" t="n">
@@ -833,7 +850,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>45505</v>
       </c>
       <c r="B21" t="n">
@@ -853,7 +870,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>45474</v>
       </c>
       <c r="B22" t="n">
@@ -873,7 +890,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>45444</v>
       </c>
       <c r="B23" t="n">
@@ -893,7 +910,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>45413</v>
       </c>
       <c r="B24" t="n">
@@ -913,7 +930,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>45383</v>
       </c>
       <c r="B25" t="n">
@@ -933,7 +950,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>45352</v>
       </c>
       <c r="B26" t="n">
@@ -953,7 +970,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>45323</v>
       </c>
       <c r="B27" t="n">
@@ -973,7 +990,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>45292</v>
       </c>
       <c r="B28" t="n">
@@ -993,7 +1010,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>45261</v>
       </c>
       <c r="B29" t="n">
@@ -1013,7 +1030,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>45231</v>
       </c>
       <c r="B30" t="n">
@@ -1033,7 +1050,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>45200</v>
       </c>
       <c r="B31" t="n">
@@ -1053,7 +1070,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>45170</v>
       </c>
       <c r="B32" t="n">
@@ -1073,7 +1090,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>45139</v>
       </c>
       <c r="B33" t="n">
@@ -1093,7 +1110,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>45108</v>
       </c>
       <c r="B34" t="n">
@@ -1113,7 +1130,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>45078</v>
       </c>
       <c r="B35" t="n">
@@ -1133,7 +1150,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>45047</v>
       </c>
       <c r="B36" t="n">
@@ -1153,7 +1170,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>45017</v>
       </c>
       <c r="B37" t="n">
@@ -1173,7 +1190,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>44986</v>
       </c>
       <c r="B38" t="n">
@@ -1193,7 +1210,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>44958</v>
       </c>
       <c r="B39" t="n">
@@ -1213,7 +1230,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>44927</v>
       </c>
       <c r="B40" t="n">
@@ -1233,7 +1250,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>44896</v>
       </c>
       <c r="B41" t="n">
@@ -1253,7 +1270,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>44866</v>
       </c>
       <c r="B42" t="n">
@@ -1273,7 +1290,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>44835</v>
       </c>
       <c r="B43" t="n">
@@ -1293,7 +1310,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>44805</v>
       </c>
       <c r="B44" t="n">
@@ -1313,7 +1330,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>44774</v>
       </c>
       <c r="B45" t="n">
@@ -1333,7 +1350,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>44743</v>
       </c>
       <c r="B46" t="n">
@@ -1353,7 +1370,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>44713</v>
       </c>
       <c r="B47" t="n">
@@ -1373,7 +1390,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>44682</v>
       </c>
       <c r="B48" t="n">
@@ -1393,7 +1410,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>44652</v>
       </c>
       <c r="B49" t="n">
@@ -1413,7 +1430,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>44621</v>
       </c>
       <c r="B50" t="n">
@@ -1433,7 +1450,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>44593</v>
       </c>
       <c r="B51" t="n">
@@ -1453,7 +1470,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>44562</v>
       </c>
       <c r="B52" t="n">
@@ -1473,7 +1490,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>44531</v>
       </c>
       <c r="B53" t="n">
@@ -1493,7 +1510,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="B54" t="n">
@@ -1513,7 +1530,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>44470</v>
       </c>
       <c r="B55" t="n">
@@ -1533,7 +1550,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>44440</v>
       </c>
       <c r="B56" t="n">
@@ -1553,7 +1570,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>44409</v>
       </c>
       <c r="B57" t="n">
@@ -1573,7 +1590,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>44378</v>
       </c>
       <c r="B58" t="n">
@@ -1593,7 +1610,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>44348</v>
       </c>
       <c r="B59" t="n">
@@ -1613,7 +1630,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>44317</v>
       </c>
       <c r="B60" t="n">
@@ -1633,7 +1650,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>44287</v>
       </c>
       <c r="B61" t="n">
@@ -1653,7 +1670,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>44256</v>
       </c>
       <c r="B62" t="n">
@@ -1673,7 +1690,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>44228</v>
       </c>
       <c r="B63" t="n">
@@ -1693,7 +1710,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="B64" t="n">
@@ -1713,7 +1730,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>44166</v>
       </c>
       <c r="B65" t="n">
@@ -1733,7 +1750,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>44136</v>
       </c>
       <c r="B66" t="n">
@@ -1753,7 +1770,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>44105</v>
       </c>
       <c r="B67" t="n">
@@ -1773,7 +1790,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>44075</v>
       </c>
       <c r="B68" t="n">
@@ -1793,7 +1810,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>44044</v>
       </c>
       <c r="B69" t="n">
@@ -1813,7 +1830,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>44013</v>
       </c>
       <c r="B70" t="n">
@@ -1833,7 +1850,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>43983</v>
       </c>
       <c r="B71" t="n">
@@ -1853,7 +1870,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>43952</v>
       </c>
       <c r="B72" t="n">
@@ -1873,7 +1890,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>43922</v>
       </c>
       <c r="B73" t="n">
@@ -1893,7 +1910,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>43891</v>
       </c>
       <c r="B74" t="n">
@@ -1913,7 +1930,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>43862</v>
       </c>
       <c r="B75" t="n">
@@ -1933,7 +1950,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="B76" t="n">
@@ -1953,7 +1970,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>43800</v>
       </c>
       <c r="B77" t="n">
@@ -1973,7 +1990,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>43770</v>
       </c>
       <c r="B78" t="n">
@@ -1993,7 +2010,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>43739</v>
       </c>
       <c r="B79" t="n">
@@ -2013,7 +2030,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>43709</v>
       </c>
       <c r="B80" t="n">
@@ -2033,7 +2050,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>43678</v>
       </c>
       <c r="B81" t="n">
@@ -2053,7 +2070,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="B82" t="n">
@@ -2073,7 +2090,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>43617</v>
       </c>
       <c r="B83" t="n">
@@ -2093,7 +2110,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>43586</v>
       </c>
       <c r="B84" t="n">
@@ -2113,7 +2130,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>43556</v>
       </c>
       <c r="B85" t="n">
@@ -2133,7 +2150,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>43525</v>
       </c>
       <c r="B86" t="n">
@@ -2153,7 +2170,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>43497</v>
       </c>
       <c r="B87" t="n">
@@ -2173,7 +2190,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="B88" t="n">
@@ -2193,7 +2210,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>43435</v>
       </c>
       <c r="B89" t="n">
@@ -2213,7 +2230,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>43405</v>
       </c>
       <c r="B90" t="n">
@@ -2233,7 +2250,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>43374</v>
       </c>
       <c r="B91" t="n">
@@ -2253,7 +2270,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>43344</v>
       </c>
       <c r="B92" t="n">
@@ -2273,7 +2290,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>43313</v>
       </c>
       <c r="B93" t="n">
@@ -2293,7 +2310,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>43282</v>
       </c>
       <c r="B94" t="n">
@@ -2313,7 +2330,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>43252</v>
       </c>
       <c r="B95" t="n">
@@ -2333,7 +2350,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>43221</v>
       </c>
       <c r="B96" t="n">
@@ -2353,7 +2370,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>43191</v>
       </c>
       <c r="B97" t="n">
@@ -2373,7 +2390,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>43160</v>
       </c>
       <c r="B98" t="n">
@@ -2393,7 +2410,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>43132</v>
       </c>
       <c r="B99" t="n">
@@ -2413,7 +2430,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>43101</v>
       </c>
       <c r="B100" t="n">
@@ -2433,7 +2450,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>43070</v>
       </c>
       <c r="B101" t="n">
@@ -2453,7 +2470,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>43040</v>
       </c>
       <c r="B102" t="n">
@@ -2473,7 +2490,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>43009</v>
       </c>
       <c r="B103" t="n">
@@ -2493,7 +2510,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>42979</v>
       </c>
       <c r="B104" t="n">
@@ -2513,7 +2530,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>42948</v>
       </c>
       <c r="B105" t="n">
@@ -2533,7 +2550,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>42917</v>
       </c>
       <c r="B106" t="n">
@@ -2553,7 +2570,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>42887</v>
       </c>
       <c r="B107" t="n">
@@ -2574,5 +2591,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add symbol column to outputs
</commit_message>
<xml_diff>
--- a/data/generated/dher_de.xlsx
+++ b/data/generated/dher_de.xlsx
@@ -135,6 +135,13 @@
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Refreshed from Yahoo Finance DHER.DE monthly history on 2026-03-11 01:41:10.
+https://finance.yahoo.com/quote/DHER.DE/history/
+Earliest reliable live month for this series: 2010-06-01.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Refreshed from Yahoo Finance DHER.DE monthly history on 2026-03-11 01:35:44.
 https://finance.yahoo.com/quote/DHER.DE/history/
@@ -434,2158 +441,2693 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>symbol</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>close</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>46082</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>18.58</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>19.14</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>16.72</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>18.07</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>9289581</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
         <v>46054</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>24.2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>26.52</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>18.86</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>19.66</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>21186525</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>22.72</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>27.26</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>21.32</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>23.6</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>18272277</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
         <v>45992</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>19.82</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>22.85</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>18.18</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>22.72</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>11401787</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
         <v>45962</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>21.85</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>21.87</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>15.73</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>20.1</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>23598116</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>24.32</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>26.26</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>21.81</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>22</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>12053573</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
         <v>45901</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>22.44</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>29.89</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>22.4</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>24.24</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>13115739</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>26</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>26.43</v>
-      </c>
-      <c r="D9" t="n">
-        <v>22.05</v>
       </c>
       <c r="E9" t="n">
         <v>22.05</v>
       </c>
       <c r="F9" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="G9" t="n">
         <v>10677376</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>23.1</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>28.28</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>21.31</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>26.29</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>20698953</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
         <v>45809</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>24.19</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>25.02</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>20.67</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>22.97</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>14678991</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>25.35</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>27.56</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>23.94</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>24.38</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>10599540</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>22.34</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>27.53</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>19.69</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>24.79</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>16778857</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
         <v>45717</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>28.11</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>30.19</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>21.59</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>21.97</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>18409643</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
         <v>45689</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>24.4</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>32.35</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>23.9</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>28.02</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>15815036</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
         <v>45658</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>27.04</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>30.34</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>24.72</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>24.97</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>12482724</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
         <v>45627</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>36.24</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>36.69</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>26</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>27.04</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>13953776</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
         <v>45597</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>38.96</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>40.76</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>35.1</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>38.74</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>10088137</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
         <v>45566</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>36.14</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>42.05</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>35.7</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>38.91</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>13265065</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
         <v>45536</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>28.29</v>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>36.46</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>26.22</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>36.22</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>17097048</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
         <v>45505</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>20.31</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>28.84</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>18.06</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>28.49</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>14774085</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
         <v>45474</v>
       </c>
-      <c r="B22" t="n">
+      <c r="C22" t="n">
         <v>22.6</v>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>23.08</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>17.35</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>20.61</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>20089181</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
         <v>45444</v>
       </c>
-      <c r="B23" t="n">
+      <c r="C23" t="n">
         <v>28.11</v>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>29.55</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>21.28</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>22.15</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>10641536</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>45413</v>
       </c>
-      <c r="B24" t="n">
+      <c r="C24" t="n">
         <v>26.3</v>
       </c>
-      <c r="C24" t="n">
+      <c r="D24" t="n">
         <v>32.48</v>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>24.27</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>27.91</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>18898771</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="B25" t="n">
+      <c r="C25" t="n">
         <v>26.8</v>
       </c>
-      <c r="C25" t="n">
+      <c r="D25" t="n">
         <v>33.93</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>24.7</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>26.4</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>26261109</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
         <v>45352</v>
       </c>
-      <c r="B26" t="n">
+      <c r="C26" t="n">
         <v>21.44</v>
       </c>
-      <c r="C26" t="n">
+      <c r="D26" t="n">
         <v>28</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
         <v>20.95</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>26.51</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>22485106</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
         <v>45323</v>
       </c>
-      <c r="B27" t="n">
+      <c r="C27" t="n">
         <v>21.1</v>
       </c>
-      <c r="C27" t="n">
+      <c r="D27" t="n">
         <v>24.15</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>14.92</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>21.36</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>43339506</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
         <v>45292</v>
       </c>
-      <c r="B28" t="n">
+      <c r="C28" t="n">
         <v>25.01</v>
       </c>
-      <c r="C28" t="n">
+      <c r="D28" t="n">
         <v>25.32</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>20.09</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>21.3</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>18096539</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
         <v>45261</v>
       </c>
-      <c r="B29" t="n">
+      <c r="C29" t="n">
         <v>28.82</v>
       </c>
-      <c r="C29" t="n">
+      <c r="D29" t="n">
         <v>32.21</v>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
         <v>23.83</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>25.01</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>14255985</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
         <v>45231</v>
       </c>
-      <c r="B30" t="n">
+      <c r="C30" t="n">
         <v>23.27</v>
       </c>
-      <c r="C30" t="n">
+      <c r="D30" t="n">
         <v>33.67</v>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>22.95</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>29.1</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>15486526</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
         <v>45200</v>
       </c>
-      <c r="B31" t="n">
+      <c r="C31" t="n">
         <v>27.42</v>
       </c>
-      <c r="C31" t="n">
+      <c r="D31" t="n">
         <v>29.45</v>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
         <v>21.73</v>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>23.97</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>13176741</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
         <v>45170</v>
       </c>
-      <c r="B32" t="n">
+      <c r="C32" t="n">
         <v>33.49</v>
       </c>
-      <c r="C32" t="n">
+      <c r="D32" t="n">
         <v>34.28</v>
       </c>
-      <c r="D32" t="n">
+      <c r="E32" t="n">
         <v>26.53</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>27.17</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>15402678</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>45139</v>
       </c>
-      <c r="B33" t="n">
+      <c r="C33" t="n">
         <v>40.9</v>
       </c>
-      <c r="C33" t="n">
+      <c r="D33" t="n">
         <v>41.17</v>
       </c>
-      <c r="D33" t="n">
+      <c r="E33" t="n">
         <v>31.25</v>
       </c>
-      <c r="E33" t="n">
+      <c r="F33" t="n">
         <v>33.72</v>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>10953100</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
         <v>45108</v>
       </c>
-      <c r="B34" t="n">
+      <c r="C34" t="n">
         <v>40.56</v>
       </c>
-      <c r="C34" t="n">
+      <c r="D34" t="n">
         <v>43.96</v>
       </c>
-      <c r="D34" t="n">
+      <c r="E34" t="n">
         <v>37.72</v>
       </c>
-      <c r="E34" t="n">
+      <c r="F34" t="n">
         <v>41.26</v>
       </c>
-      <c r="F34" t="n">
+      <c r="G34" t="n">
         <v>11343421</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
         <v>45078</v>
       </c>
-      <c r="B35" t="n">
+      <c r="C35" t="n">
         <v>35.29</v>
       </c>
-      <c r="C35" t="n">
+      <c r="D35" t="n">
         <v>40.4</v>
       </c>
-      <c r="D35" t="n">
+      <c r="E35" t="n">
         <v>33.7</v>
       </c>
-      <c r="E35" t="n">
+      <c r="F35" t="n">
         <v>40.4</v>
       </c>
-      <c r="F35" t="n">
+      <c r="G35" t="n">
         <v>12250976</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
         <v>45047</v>
       </c>
-      <c r="B36" t="n">
+      <c r="C36" t="n">
         <v>36.13</v>
       </c>
-      <c r="C36" t="n">
+      <c r="D36" t="n">
         <v>41.1</v>
       </c>
-      <c r="D36" t="n">
+      <c r="E36" t="n">
         <v>34.82</v>
       </c>
-      <c r="E36" t="n">
+      <c r="F36" t="n">
         <v>35</v>
       </c>
-      <c r="F36" t="n">
+      <c r="G36" t="n">
         <v>11506441</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
         <v>45017</v>
       </c>
-      <c r="B37" t="n">
+      <c r="C37" t="n">
         <v>31.37</v>
       </c>
-      <c r="C37" t="n">
+      <c r="D37" t="n">
         <v>36.72</v>
       </c>
-      <c r="D37" t="n">
+      <c r="E37" t="n">
         <v>29.31</v>
       </c>
-      <c r="E37" t="n">
+      <c r="F37" t="n">
         <v>36.13</v>
       </c>
-      <c r="F37" t="n">
+      <c r="G37" t="n">
         <v>11942550</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
         <v>44986</v>
       </c>
-      <c r="B38" t="n">
+      <c r="C38" t="n">
         <v>38.81</v>
       </c>
-      <c r="C38" t="n">
+      <c r="D38" t="n">
         <v>39.44</v>
       </c>
-      <c r="D38" t="n">
+      <c r="E38" t="n">
         <v>29.34</v>
       </c>
-      <c r="E38" t="n">
+      <c r="F38" t="n">
         <v>31.37</v>
       </c>
-      <c r="F38" t="n">
+      <c r="G38" t="n">
         <v>14924644</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
         <v>44958</v>
       </c>
-      <c r="B39" t="n">
+      <c r="C39" t="n">
         <v>55.32</v>
       </c>
-      <c r="C39" t="n">
+      <c r="D39" t="n">
         <v>57.82</v>
       </c>
-      <c r="D39" t="n">
+      <c r="E39" t="n">
         <v>37.05</v>
       </c>
-      <c r="E39" t="n">
+      <c r="F39" t="n">
         <v>38.19</v>
       </c>
-      <c r="F39" t="n">
+      <c r="G39" t="n">
         <v>16021794</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
         <v>44927</v>
       </c>
-      <c r="B40" t="n">
+      <c r="C40" t="n">
         <v>45.1</v>
       </c>
-      <c r="C40" t="n">
+      <c r="D40" t="n">
         <v>55.88</v>
       </c>
-      <c r="D40" t="n">
+      <c r="E40" t="n">
         <v>43.43</v>
       </c>
-      <c r="E40" t="n">
+      <c r="F40" t="n">
         <v>55.22</v>
       </c>
-      <c r="F40" t="n">
+      <c r="G40" t="n">
         <v>12174820</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
         <v>44896</v>
       </c>
-      <c r="B41" t="n">
+      <c r="C41" t="n">
         <v>42.76</v>
       </c>
-      <c r="C41" t="n">
+      <c r="D41" t="n">
         <v>46.61</v>
       </c>
-      <c r="D41" t="n">
+      <c r="E41" t="n">
         <v>39.1</v>
       </c>
-      <c r="E41" t="n">
+      <c r="F41" t="n">
         <v>44.78</v>
       </c>
-      <c r="F41" t="n">
+      <c r="G41" t="n">
         <v>10675975</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
         <v>44866</v>
       </c>
-      <c r="B42" t="n">
+      <c r="C42" t="n">
         <v>34.27</v>
       </c>
-      <c r="C42" t="n">
+      <c r="D42" t="n">
         <v>46.91</v>
       </c>
-      <c r="D42" t="n">
+      <c r="E42" t="n">
         <v>32.37</v>
       </c>
-      <c r="E42" t="n">
+      <c r="F42" t="n">
         <v>40.97</v>
       </c>
-      <c r="F42" t="n">
+      <c r="G42" t="n">
         <v>18693436</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
         <v>44835</v>
       </c>
-      <c r="B43" t="n">
+      <c r="C43" t="n">
         <v>37.78</v>
       </c>
-      <c r="C43" t="n">
+      <c r="D43" t="n">
         <v>40.91</v>
       </c>
-      <c r="D43" t="n">
+      <c r="E43" t="n">
         <v>30.61</v>
       </c>
-      <c r="E43" t="n">
+      <c r="F43" t="n">
         <v>33.35</v>
       </c>
-      <c r="F43" t="n">
+      <c r="G43" t="n">
         <v>13646243</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
         <v>44805</v>
       </c>
-      <c r="B44" t="n">
+      <c r="C44" t="n">
         <v>40.84</v>
       </c>
-      <c r="C44" t="n">
+      <c r="D44" t="n">
         <v>50.58</v>
       </c>
-      <c r="D44" t="n">
+      <c r="E44" t="n">
         <v>36.04</v>
       </c>
-      <c r="E44" t="n">
+      <c r="F44" t="n">
         <v>37.94</v>
       </c>
-      <c r="F44" t="n">
+      <c r="G44" t="n">
         <v>16584790</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
         <v>44774</v>
       </c>
-      <c r="B45" t="n">
+      <c r="C45" t="n">
         <v>46.82</v>
       </c>
-      <c r="C45" t="n">
+      <c r="D45" t="n">
         <v>57.16</v>
-      </c>
-      <c r="D45" t="n">
-        <v>41.5</v>
       </c>
       <c r="E45" t="n">
         <v>41.5</v>
       </c>
       <c r="F45" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="G45" t="n">
         <v>16666747</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
         <v>44743</v>
       </c>
-      <c r="B46" t="n">
+      <c r="C46" t="n">
         <v>35.47</v>
       </c>
-      <c r="C46" t="n">
+      <c r="D46" t="n">
         <v>49.97</v>
       </c>
-      <c r="D46" t="n">
+      <c r="E46" t="n">
         <v>33.66</v>
       </c>
-      <c r="E46" t="n">
+      <c r="F46" t="n">
         <v>46.91</v>
       </c>
-      <c r="F46" t="n">
+      <c r="G46" t="n">
         <v>21978974</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
         <v>44713</v>
       </c>
-      <c r="B47" t="n">
+      <c r="C47" t="n">
         <v>35.51</v>
       </c>
-      <c r="C47" t="n">
+      <c r="D47" t="n">
         <v>41.57</v>
       </c>
-      <c r="D47" t="n">
+      <c r="E47" t="n">
         <v>31.02</v>
       </c>
-      <c r="E47" t="n">
+      <c r="F47" t="n">
         <v>35.77</v>
       </c>
-      <c r="F47" t="n">
+      <c r="G47" t="n">
         <v>35787423</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
         <v>44682</v>
       </c>
-      <c r="B48" t="n">
+      <c r="C48" t="n">
         <v>33.84</v>
       </c>
-      <c r="C48" t="n">
+      <c r="D48" t="n">
         <v>37.22</v>
       </c>
-      <c r="D48" t="n">
+      <c r="E48" t="n">
         <v>23.88</v>
       </c>
-      <c r="E48" t="n">
+      <c r="F48" t="n">
         <v>35.74</v>
       </c>
-      <c r="F48" t="n">
+      <c r="G48" t="n">
         <v>27230838</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
         <v>44652</v>
       </c>
-      <c r="B49" t="n">
+      <c r="C49" t="n">
         <v>40</v>
       </c>
-      <c r="C49" t="n">
+      <c r="D49" t="n">
         <v>49.11</v>
       </c>
-      <c r="D49" t="n">
+      <c r="E49" t="n">
         <v>26.18</v>
       </c>
-      <c r="E49" t="n">
+      <c r="F49" t="n">
         <v>33.84</v>
       </c>
-      <c r="F49" t="n">
+      <c r="G49" t="n">
         <v>34856933</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
         <v>44621</v>
       </c>
-      <c r="B50" t="n">
+      <c r="C50" t="n">
         <v>48.39</v>
       </c>
-      <c r="C50" t="n">
+      <c r="D50" t="n">
         <v>50.28</v>
       </c>
-      <c r="D50" t="n">
+      <c r="E50" t="n">
         <v>36.45</v>
       </c>
-      <c r="E50" t="n">
+      <c r="F50" t="n">
         <v>39.86</v>
       </c>
-      <c r="F50" t="n">
+      <c r="G50" t="n">
         <v>40171110</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
         <v>44593</v>
       </c>
-      <c r="B51" t="n">
+      <c r="C51" t="n">
         <v>68.5</v>
       </c>
-      <c r="C51" t="n">
+      <c r="D51" t="n">
         <v>72.31999999999999</v>
       </c>
-      <c r="D51" t="n">
+      <c r="E51" t="n">
         <v>38.75</v>
       </c>
-      <c r="E51" t="n">
+      <c r="F51" t="n">
         <v>47.81</v>
       </c>
-      <c r="F51" t="n">
+      <c r="G51" t="n">
         <v>50126389</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>44562</v>
       </c>
-      <c r="B52" t="n">
+      <c r="C52" t="n">
         <v>97.7</v>
       </c>
-      <c r="C52" t="n">
+      <c r="D52" t="n">
         <v>100.45</v>
       </c>
-      <c r="D52" t="n">
+      <c r="E52" t="n">
         <v>62.44</v>
       </c>
-      <c r="E52" t="n">
+      <c r="F52" t="n">
         <v>67.92</v>
       </c>
-      <c r="F52" t="n">
+      <c r="G52" t="n">
         <v>19514559</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
         <v>44531</v>
       </c>
-      <c r="B53" t="n">
+      <c r="C53" t="n">
         <v>118.05</v>
       </c>
-      <c r="C53" t="n">
+      <c r="D53" t="n">
         <v>118.25</v>
       </c>
-      <c r="D53" t="n">
+      <c r="E53" t="n">
         <v>86.92</v>
       </c>
-      <c r="E53" t="n">
+      <c r="F53" t="n">
         <v>98</v>
       </c>
-      <c r="F53" t="n">
+      <c r="G53" t="n">
         <v>13609385</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>44501</v>
       </c>
-      <c r="B54" t="n">
+      <c r="C54" t="n">
         <v>107.9</v>
       </c>
-      <c r="C54" t="n">
+      <c r="D54" t="n">
         <v>131.5</v>
       </c>
-      <c r="D54" t="n">
+      <c r="E54" t="n">
         <v>105.55</v>
       </c>
-      <c r="E54" t="n">
+      <c r="F54" t="n">
         <v>117.7</v>
       </c>
-      <c r="F54" t="n">
+      <c r="G54" t="n">
         <v>11337027</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>44470</v>
       </c>
-      <c r="B55" t="n">
+      <c r="C55" t="n">
         <v>110.1</v>
       </c>
-      <c r="C55" t="n">
+      <c r="D55" t="n">
         <v>119.1</v>
       </c>
-      <c r="D55" t="n">
+      <c r="E55" t="n">
         <v>101.65</v>
       </c>
-      <c r="E55" t="n">
+      <c r="F55" t="n">
         <v>107.55</v>
       </c>
-      <c r="F55" t="n">
+      <c r="G55" t="n">
         <v>9383348</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
         <v>44440</v>
       </c>
-      <c r="B56" t="n">
+      <c r="C56" t="n">
         <v>123.8</v>
       </c>
-      <c r="C56" t="n">
+      <c r="D56" t="n">
         <v>134.95</v>
       </c>
-      <c r="D56" t="n">
+      <c r="E56" t="n">
         <v>110.25</v>
       </c>
-      <c r="E56" t="n">
+      <c r="F56" t="n">
         <v>110.45</v>
       </c>
-      <c r="F56" t="n">
+      <c r="G56" t="n">
         <v>9992438</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
         <v>44409</v>
       </c>
-      <c r="B57" t="n">
+      <c r="C57" t="n">
         <v>126.45</v>
       </c>
-      <c r="C57" t="n">
+      <c r="D57" t="n">
         <v>132.85</v>
       </c>
-      <c r="D57" t="n">
+      <c r="E57" t="n">
         <v>112.05</v>
       </c>
-      <c r="E57" t="n">
+      <c r="F57" t="n">
         <v>122.6</v>
       </c>
-      <c r="F57" t="n">
+      <c r="G57" t="n">
         <v>10152987</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="B58" t="n">
+      <c r="C58" t="n">
         <v>112.35</v>
       </c>
-      <c r="C58" t="n">
+      <c r="D58" t="n">
         <v>130</v>
       </c>
-      <c r="D58" t="n">
+      <c r="E58" t="n">
         <v>110.6</v>
       </c>
-      <c r="E58" t="n">
+      <c r="F58" t="n">
         <v>126.2</v>
       </c>
-      <c r="F58" t="n">
+      <c r="G58" t="n">
         <v>8725365</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
         <v>44348</v>
       </c>
-      <c r="B59" t="n">
+      <c r="C59" t="n">
         <v>112.95</v>
       </c>
-      <c r="C59" t="n">
+      <c r="D59" t="n">
         <v>115.65</v>
       </c>
-      <c r="D59" t="n">
+      <c r="E59" t="n">
         <v>105.15</v>
       </c>
-      <c r="E59" t="n">
+      <c r="F59" t="n">
         <v>111.4</v>
       </c>
-      <c r="F59" t="n">
+      <c r="G59" t="n">
         <v>10836677</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
         <v>44317</v>
       </c>
-      <c r="B60" t="n">
+      <c r="C60" t="n">
         <v>131.95</v>
       </c>
-      <c r="C60" t="n">
+      <c r="D60" t="n">
         <v>133.1</v>
       </c>
-      <c r="D60" t="n">
+      <c r="E60" t="n">
         <v>101.3</v>
       </c>
-      <c r="E60" t="n">
+      <c r="F60" t="n">
         <v>112.5</v>
       </c>
-      <c r="F60" t="n">
+      <c r="G60" t="n">
         <v>16716704</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>44287</v>
       </c>
-      <c r="B61" t="n">
+      <c r="C61" t="n">
         <v>113.75</v>
       </c>
-      <c r="C61" t="n">
+      <c r="D61" t="n">
         <v>141.95</v>
       </c>
-      <c r="D61" t="n">
+      <c r="E61" t="n">
         <v>111.85</v>
       </c>
-      <c r="E61" t="n">
+      <c r="F61" t="n">
         <v>132.05</v>
       </c>
-      <c r="F61" t="n">
+      <c r="G61" t="n">
         <v>11840909</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
         <v>44256</v>
       </c>
-      <c r="B62" t="n">
+      <c r="C62" t="n">
         <v>107.5</v>
       </c>
-      <c r="C62" t="n">
+      <c r="D62" t="n">
         <v>113.65</v>
       </c>
-      <c r="D62" t="n">
+      <c r="E62" t="n">
         <v>100.05</v>
       </c>
-      <c r="E62" t="n">
+      <c r="F62" t="n">
         <v>110.5</v>
       </c>
-      <c r="F62" t="n">
+      <c r="G62" t="n">
         <v>18994357</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
         <v>44228</v>
       </c>
-      <c r="B63" t="n">
+      <c r="C63" t="n">
         <v>126.5</v>
       </c>
-      <c r="C63" t="n">
+      <c r="D63" t="n">
         <v>134.45</v>
       </c>
-      <c r="D63" t="n">
+      <c r="E63" t="n">
         <v>104.8</v>
       </c>
-      <c r="E63" t="n">
+      <c r="F63" t="n">
         <v>105.7</v>
       </c>
-      <c r="F63" t="n">
+      <c r="G63" t="n">
         <v>11765421</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
         <v>44197</v>
       </c>
-      <c r="B64" t="n">
+      <c r="C64" t="n">
         <v>127</v>
       </c>
-      <c r="C64" t="n">
+      <c r="D64" t="n">
         <v>145.4</v>
       </c>
-      <c r="D64" t="n">
+      <c r="E64" t="n">
         <v>121.4</v>
       </c>
-      <c r="E64" t="n">
+      <c r="F64" t="n">
         <v>125.5</v>
       </c>
-      <c r="F64" t="n">
+      <c r="G64" t="n">
         <v>15069678</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
         <v>44166</v>
       </c>
-      <c r="B65" t="n">
+      <c r="C65" t="n">
         <v>101.8</v>
       </c>
-      <c r="C65" t="n">
+      <c r="D65" t="n">
         <v>132.1</v>
       </c>
-      <c r="D65" t="n">
+      <c r="E65" t="n">
         <v>97.38</v>
       </c>
-      <c r="E65" t="n">
+      <c r="F65" t="n">
         <v>127</v>
       </c>
-      <c r="F65" t="n">
+      <c r="G65" t="n">
         <v>12074860</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
         <v>44136</v>
       </c>
-      <c r="B66" t="n">
+      <c r="C66" t="n">
         <v>98.5</v>
       </c>
-      <c r="C66" t="n">
+      <c r="D66" t="n">
         <v>116.65</v>
       </c>
-      <c r="D66" t="n">
+      <c r="E66" t="n">
         <v>91</v>
       </c>
-      <c r="E66" t="n">
+      <c r="F66" t="n">
         <v>101.25</v>
       </c>
-      <c r="F66" t="n">
+      <c r="G66" t="n">
         <v>20451033</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
         <v>44105</v>
       </c>
-      <c r="B67" t="n">
+      <c r="C67" t="n">
         <v>98.26000000000001</v>
       </c>
-      <c r="C67" t="n">
+      <c r="D67" t="n">
         <v>104.85</v>
       </c>
-      <c r="D67" t="n">
+      <c r="E67" t="n">
         <v>90.59999999999999</v>
       </c>
-      <c r="E67" t="n">
+      <c r="F67" t="n">
         <v>98.78</v>
       </c>
-      <c r="F67" t="n">
+      <c r="G67" t="n">
         <v>11623884</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
         <v>44075</v>
       </c>
-      <c r="B68" t="n">
+      <c r="C68" t="n">
         <v>91.34</v>
       </c>
-      <c r="C68" t="n">
+      <c r="D68" t="n">
         <v>99.7</v>
       </c>
-      <c r="D68" t="n">
+      <c r="E68" t="n">
         <v>85.23999999999999</v>
       </c>
-      <c r="E68" t="n">
+      <c r="F68" t="n">
         <v>98.12</v>
       </c>
-      <c r="F68" t="n">
+      <c r="G68" t="n">
         <v>11812518</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
         <v>44044</v>
       </c>
-      <c r="B69" t="n">
+      <c r="C69" t="n">
         <v>98.5</v>
       </c>
-      <c r="C69" t="n">
+      <c r="D69" t="n">
         <v>105</v>
       </c>
-      <c r="D69" t="n">
+      <c r="E69" t="n">
         <v>86</v>
       </c>
-      <c r="E69" t="n">
+      <c r="F69" t="n">
         <v>90.02</v>
       </c>
-      <c r="F69" t="n">
+      <c r="G69" t="n">
         <v>13195088</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
         <v>44013</v>
       </c>
-      <c r="B70" t="n">
+      <c r="C70" t="n">
         <v>93</v>
       </c>
-      <c r="C70" t="n">
+      <c r="D70" t="n">
         <v>106.2</v>
       </c>
-      <c r="D70" t="n">
+      <c r="E70" t="n">
         <v>89.2</v>
       </c>
-      <c r="E70" t="n">
+      <c r="F70" t="n">
         <v>97.76000000000001</v>
       </c>
-      <c r="F70" t="n">
+      <c r="G70" t="n">
         <v>11155145</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
         <v>43983</v>
       </c>
-      <c r="B71" t="n">
+      <c r="C71" t="n">
         <v>86.18000000000001</v>
       </c>
-      <c r="C71" t="n">
+      <c r="D71" t="n">
         <v>96.22</v>
       </c>
-      <c r="D71" t="n">
+      <c r="E71" t="n">
         <v>82.08</v>
       </c>
-      <c r="E71" t="n">
+      <c r="F71" t="n">
         <v>90.95999999999999</v>
       </c>
-      <c r="F71" t="n">
+      <c r="G71" t="n">
         <v>10155901</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>43952</v>
       </c>
-      <c r="B72" t="n">
+      <c r="C72" t="n">
         <v>77</v>
       </c>
-      <c r="C72" t="n">
+      <c r="D72" t="n">
         <v>91.98</v>
       </c>
-      <c r="D72" t="n">
+      <c r="E72" t="n">
         <v>75.04000000000001</v>
       </c>
-      <c r="E72" t="n">
+      <c r="F72" t="n">
         <v>86.18000000000001</v>
       </c>
-      <c r="F72" t="n">
+      <c r="G72" t="n">
         <v>10420653</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
         <v>43922</v>
       </c>
-      <c r="B73" t="n">
+      <c r="C73" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="C73" t="n">
+      <c r="D73" t="n">
         <v>81.62</v>
       </c>
-      <c r="D73" t="n">
+      <c r="E73" t="n">
         <v>58.54</v>
       </c>
-      <c r="E73" t="n">
+      <c r="F73" t="n">
         <v>77</v>
       </c>
-      <c r="F73" t="n">
+      <c r="G73" t="n">
         <v>8602825</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
         <v>43891</v>
       </c>
-      <c r="B74" t="n">
+      <c r="C74" t="n">
         <v>72</v>
       </c>
-      <c r="C74" t="n">
+      <c r="D74" t="n">
         <v>73.26000000000001</v>
       </c>
-      <c r="D74" t="n">
+      <c r="E74" t="n">
         <v>50.18</v>
       </c>
-      <c r="E74" t="n">
+      <c r="F74" t="n">
         <v>67.95999999999999</v>
       </c>
-      <c r="F74" t="n">
+      <c r="G74" t="n">
         <v>16883690</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
         <v>43862</v>
       </c>
-      <c r="B75" t="n">
+      <c r="C75" t="n">
         <v>69.72</v>
       </c>
-      <c r="C75" t="n">
+      <c r="D75" t="n">
         <v>81.62</v>
       </c>
-      <c r="D75" t="n">
+      <c r="E75" t="n">
         <v>64.5</v>
       </c>
-      <c r="E75" t="n">
+      <c r="F75" t="n">
         <v>68</v>
       </c>
-      <c r="F75" t="n">
+      <c r="G75" t="n">
         <v>11185012</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
         <v>43831</v>
       </c>
-      <c r="B76" t="n">
+      <c r="C76" t="n">
         <v>70.56</v>
       </c>
-      <c r="C76" t="n">
+      <c r="D76" t="n">
         <v>72.18000000000001</v>
       </c>
-      <c r="D76" t="n">
+      <c r="E76" t="n">
         <v>64.58</v>
       </c>
-      <c r="E76" t="n">
+      <c r="F76" t="n">
         <v>69.62</v>
       </c>
-      <c r="F76" t="n">
+      <c r="G76" t="n">
         <v>10597357</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
         <v>43800</v>
       </c>
-      <c r="B77" t="n">
+      <c r="C77" t="n">
         <v>47.79</v>
       </c>
-      <c r="C77" t="n">
+      <c r="D77" t="n">
         <v>71.72</v>
       </c>
-      <c r="D77" t="n">
+      <c r="E77" t="n">
         <v>47.51</v>
       </c>
-      <c r="E77" t="n">
+      <c r="F77" t="n">
         <v>70.56</v>
       </c>
-      <c r="F77" t="n">
+      <c r="G77" t="n">
         <v>10678792</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
         <v>43770</v>
       </c>
-      <c r="B78" t="n">
+      <c r="C78" t="n">
         <v>41.73</v>
       </c>
-      <c r="C78" t="n">
+      <c r="D78" t="n">
         <v>48.52</v>
       </c>
-      <c r="D78" t="n">
+      <c r="E78" t="n">
         <v>40.47</v>
       </c>
-      <c r="E78" t="n">
+      <c r="F78" t="n">
         <v>48</v>
       </c>
-      <c r="F78" t="n">
+      <c r="G78" t="n">
         <v>7118671</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
         <v>43739</v>
       </c>
-      <c r="B79" t="n">
+      <c r="C79" t="n">
         <v>40.74</v>
       </c>
-      <c r="C79" t="n">
+      <c r="D79" t="n">
         <v>46</v>
       </c>
-      <c r="D79" t="n">
+      <c r="E79" t="n">
         <v>38.59</v>
       </c>
-      <c r="E79" t="n">
+      <c r="F79" t="n">
         <v>42.03</v>
       </c>
-      <c r="F79" t="n">
+      <c r="G79" t="n">
         <v>9270326</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
         <v>43709</v>
       </c>
-      <c r="B80" t="n">
+      <c r="C80" t="n">
         <v>46.2</v>
       </c>
-      <c r="C80" t="n">
+      <c r="D80" t="n">
         <v>48.79</v>
       </c>
-      <c r="D80" t="n">
+      <c r="E80" t="n">
         <v>40.51</v>
       </c>
-      <c r="E80" t="n">
+      <c r="F80" t="n">
         <v>40.76</v>
       </c>
-      <c r="F80" t="n">
+      <c r="G80" t="n">
         <v>7720201</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
         <v>43678</v>
       </c>
-      <c r="B81" t="n">
+      <c r="C81" t="n">
         <v>43.8</v>
       </c>
-      <c r="C81" t="n">
+      <c r="D81" t="n">
         <v>47.05</v>
       </c>
-      <c r="D81" t="n">
+      <c r="E81" t="n">
         <v>41.76</v>
       </c>
-      <c r="E81" t="n">
+      <c r="F81" t="n">
         <v>45.96</v>
       </c>
-      <c r="F81" t="n">
+      <c r="G81" t="n">
         <v>8322155</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
         <v>43647</v>
       </c>
-      <c r="B82" t="n">
+      <c r="C82" t="n">
         <v>40.43</v>
       </c>
-      <c r="C82" t="n">
+      <c r="D82" t="n">
         <v>44.34</v>
       </c>
-      <c r="D82" t="n">
+      <c r="E82" t="n">
         <v>38.45</v>
       </c>
-      <c r="E82" t="n">
+      <c r="F82" t="n">
         <v>43.58</v>
       </c>
-      <c r="F82" t="n">
+      <c r="G82" t="n">
         <v>8828979</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
         <v>43617</v>
       </c>
-      <c r="B83" t="n">
+      <c r="C83" t="n">
         <v>38.45</v>
       </c>
-      <c r="C83" t="n">
+      <c r="D83" t="n">
         <v>43.28</v>
       </c>
-      <c r="D83" t="n">
+      <c r="E83" t="n">
         <v>36.89</v>
       </c>
-      <c r="E83" t="n">
+      <c r="F83" t="n">
         <v>39.89</v>
       </c>
-      <c r="F83" t="n">
+      <c r="G83" t="n">
         <v>8093269</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
         <v>43586</v>
       </c>
-      <c r="B84" t="n">
+      <c r="C84" t="n">
         <v>41.09</v>
       </c>
-      <c r="C84" t="n">
+      <c r="D84" t="n">
         <v>43</v>
       </c>
-      <c r="D84" t="n">
+      <c r="E84" t="n">
         <v>37.64</v>
       </c>
-      <c r="E84" t="n">
+      <c r="F84" t="n">
         <v>38.55</v>
       </c>
-      <c r="F84" t="n">
+      <c r="G84" t="n">
         <v>10181834</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
         <v>43556</v>
       </c>
-      <c r="B85" t="n">
+      <c r="C85" t="n">
         <v>32.49</v>
       </c>
-      <c r="C85" t="n">
+      <c r="D85" t="n">
         <v>41.28</v>
       </c>
-      <c r="D85" t="n">
+      <c r="E85" t="n">
         <v>32.37</v>
       </c>
-      <c r="E85" t="n">
+      <c r="F85" t="n">
         <v>41.09</v>
       </c>
-      <c r="F85" t="n">
+      <c r="G85" t="n">
         <v>9315017</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>43525</v>
       </c>
-      <c r="B86" t="n">
+      <c r="C86" t="n">
         <v>34.3</v>
       </c>
-      <c r="C86" t="n">
+      <c r="D86" t="n">
         <v>35.9</v>
       </c>
-      <c r="D86" t="n">
+      <c r="E86" t="n">
         <v>31.5</v>
       </c>
-      <c r="E86" t="n">
+      <c r="F86" t="n">
         <v>32.2</v>
       </c>
-      <c r="F86" t="n">
+      <c r="G86" t="n">
         <v>6714007</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
         <v>43497</v>
       </c>
-      <c r="B87" t="n">
+      <c r="C87" t="n">
         <v>32.3</v>
       </c>
-      <c r="C87" t="n">
+      <c r="D87" t="n">
         <v>36.94</v>
       </c>
-      <c r="D87" t="n">
+      <c r="E87" t="n">
         <v>31.26</v>
       </c>
-      <c r="E87" t="n">
+      <c r="F87" t="n">
         <v>34.08</v>
       </c>
-      <c r="F87" t="n">
+      <c r="G87" t="n">
         <v>6907445</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
         <v>43466</v>
       </c>
-      <c r="B88" t="n">
+      <c r="C88" t="n">
         <v>32.5</v>
       </c>
-      <c r="C88" t="n">
+      <c r="D88" t="n">
         <v>34</v>
       </c>
-      <c r="D88" t="n">
+      <c r="E88" t="n">
         <v>29</v>
       </c>
-      <c r="E88" t="n">
+      <c r="F88" t="n">
         <v>32.2</v>
       </c>
-      <c r="F88" t="n">
+      <c r="G88" t="n">
         <v>7050238</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
         <v>43435</v>
       </c>
-      <c r="B89" t="n">
+      <c r="C89" t="n">
         <v>33.38</v>
       </c>
-      <c r="C89" t="n">
+      <c r="D89" t="n">
         <v>34.6</v>
       </c>
-      <c r="D89" t="n">
+      <c r="E89" t="n">
         <v>27.48</v>
       </c>
-      <c r="E89" t="n">
+      <c r="F89" t="n">
         <v>32.5</v>
       </c>
-      <c r="F89" t="n">
+      <c r="G89" t="n">
         <v>6852785</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
         <v>43405</v>
       </c>
-      <c r="B90" t="n">
+      <c r="C90" t="n">
         <v>35.38</v>
       </c>
-      <c r="C90" t="n">
+      <c r="D90" t="n">
         <v>39.64</v>
       </c>
-      <c r="D90" t="n">
+      <c r="E90" t="n">
         <v>30.24</v>
       </c>
-      <c r="E90" t="n">
+      <c r="F90" t="n">
         <v>32.14</v>
       </c>
-      <c r="F90" t="n">
+      <c r="G90" t="n">
         <v>7799862</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n">
         <v>43374</v>
       </c>
-      <c r="B91" t="n">
+      <c r="C91" t="n">
         <v>41.22</v>
       </c>
-      <c r="C91" t="n">
+      <c r="D91" t="n">
         <v>41.86</v>
       </c>
-      <c r="D91" t="n">
+      <c r="E91" t="n">
         <v>32.84</v>
       </c>
-      <c r="E91" t="n">
+      <c r="F91" t="n">
         <v>35.64</v>
       </c>
-      <c r="F91" t="n">
+      <c r="G91" t="n">
         <v>8848554</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n">
         <v>43344</v>
       </c>
-      <c r="B92" t="n">
+      <c r="C92" t="n">
         <v>47.5</v>
       </c>
-      <c r="C92" t="n">
+      <c r="D92" t="n">
         <v>47.68</v>
       </c>
-      <c r="D92" t="n">
+      <c r="E92" t="n">
         <v>41.16</v>
       </c>
-      <c r="E92" t="n">
+      <c r="F92" t="n">
         <v>41.42</v>
       </c>
-      <c r="F92" t="n">
+      <c r="G92" t="n">
         <v>7242977</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n">
         <v>43313</v>
       </c>
-      <c r="B93" t="n">
+      <c r="C93" t="n">
         <v>48.62</v>
       </c>
-      <c r="C93" t="n">
+      <c r="D93" t="n">
         <v>49.88</v>
       </c>
-      <c r="D93" t="n">
+      <c r="E93" t="n">
         <v>44.48</v>
       </c>
-      <c r="E93" t="n">
+      <c r="F93" t="n">
         <v>47.46</v>
       </c>
-      <c r="F93" t="n">
+      <c r="G93" t="n">
         <v>7985225</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n">
         <v>43282</v>
       </c>
-      <c r="B94" t="n">
+      <c r="C94" t="n">
         <v>45.48</v>
       </c>
-      <c r="C94" t="n">
+      <c r="D94" t="n">
         <v>52.35</v>
       </c>
-      <c r="D94" t="n">
+      <c r="E94" t="n">
         <v>45.3</v>
       </c>
-      <c r="E94" t="n">
+      <c r="F94" t="n">
         <v>48.58</v>
       </c>
-      <c r="F94" t="n">
+      <c r="G94" t="n">
         <v>7538294</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n">
         <v>43252</v>
       </c>
-      <c r="B95" t="n">
+      <c r="C95" t="n">
         <v>38.72</v>
       </c>
-      <c r="C95" t="n">
+      <c r="D95" t="n">
         <v>46</v>
       </c>
-      <c r="D95" t="n">
+      <c r="E95" t="n">
         <v>38.72</v>
       </c>
-      <c r="E95" t="n">
+      <c r="F95" t="n">
         <v>45.58</v>
       </c>
-      <c r="F95" t="n">
+      <c r="G95" t="n">
         <v>11851069</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
         <v>43221</v>
       </c>
-      <c r="B96" t="n">
+      <c r="C96" t="n">
         <v>39.6</v>
       </c>
-      <c r="C96" t="n">
+      <c r="D96" t="n">
         <v>40.96</v>
       </c>
-      <c r="D96" t="n">
+      <c r="E96" t="n">
         <v>37.78</v>
       </c>
-      <c r="E96" t="n">
+      <c r="F96" t="n">
         <v>39.32</v>
       </c>
-      <c r="F96" t="n">
+      <c r="G96" t="n">
         <v>16054415</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n">
         <v>43191</v>
       </c>
-      <c r="B97" t="n">
+      <c r="C97" t="n">
         <v>39.3</v>
       </c>
-      <c r="C97" t="n">
+      <c r="D97" t="n">
         <v>41.2</v>
       </c>
-      <c r="D97" t="n">
+      <c r="E97" t="n">
         <v>37.28</v>
       </c>
-      <c r="E97" t="n">
+      <c r="F97" t="n">
         <v>39.6</v>
       </c>
-      <c r="F97" t="n">
+      <c r="G97" t="n">
         <v>5644160</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n">
         <v>43160</v>
       </c>
-      <c r="B98" t="n">
+      <c r="C98" t="n">
         <v>35.88</v>
       </c>
-      <c r="C98" t="n">
+      <c r="D98" t="n">
         <v>40.46</v>
       </c>
-      <c r="D98" t="n">
+      <c r="E98" t="n">
         <v>35.3</v>
       </c>
-      <c r="E98" t="n">
+      <c r="F98" t="n">
         <v>39.3</v>
       </c>
-      <c r="F98" t="n">
+      <c r="G98" t="n">
         <v>8319206</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n">
         <v>43132</v>
       </c>
-      <c r="B99" t="n">
+      <c r="C99" t="n">
         <v>34.84</v>
       </c>
-      <c r="C99" t="n">
+      <c r="D99" t="n">
         <v>36.68</v>
       </c>
-      <c r="D99" t="n">
+      <c r="E99" t="n">
         <v>30.4</v>
       </c>
-      <c r="E99" t="n">
+      <c r="F99" t="n">
         <v>36</v>
       </c>
-      <c r="F99" t="n">
+      <c r="G99" t="n">
         <v>5384916</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n">
         <v>43101</v>
       </c>
-      <c r="B100" t="n">
+      <c r="C100" t="n">
         <v>33</v>
       </c>
-      <c r="C100" t="n">
+      <c r="D100" t="n">
         <v>35.32</v>
       </c>
-      <c r="D100" t="n">
+      <c r="E100" t="n">
         <v>31.4</v>
       </c>
-      <c r="E100" t="n">
+      <c r="F100" t="n">
         <v>34.56</v>
       </c>
-      <c r="F100" t="n">
+      <c r="G100" t="n">
         <v>5801286</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n">
         <v>43070</v>
       </c>
-      <c r="B101" t="n">
+      <c r="C101" t="n">
         <v>39.38</v>
       </c>
-      <c r="C101" t="n">
+      <c r="D101" t="n">
         <v>39.95</v>
       </c>
-      <c r="D101" t="n">
+      <c r="E101" t="n">
         <v>32.22</v>
       </c>
-      <c r="E101" t="n">
+      <c r="F101" t="n">
         <v>33</v>
       </c>
-      <c r="F101" t="n">
+      <c r="G101" t="n">
         <v>4389578</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
         <v>43040</v>
       </c>
-      <c r="B102" t="n">
+      <c r="C102" t="n">
         <v>37.49</v>
       </c>
-      <c r="C102" t="n">
+      <c r="D102" t="n">
         <v>39.75</v>
       </c>
-      <c r="D102" t="n">
+      <c r="E102" t="n">
         <v>36.33</v>
       </c>
-      <c r="E102" t="n">
+      <c r="F102" t="n">
         <v>38.9</v>
       </c>
-      <c r="F102" t="n">
+      <c r="G102" t="n">
         <v>1097242</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n">
         <v>43009</v>
       </c>
-      <c r="B103" t="n">
+      <c r="C103" t="n">
         <v>33.78</v>
       </c>
-      <c r="C103" t="n">
+      <c r="D103" t="n">
         <v>38.4</v>
       </c>
-      <c r="D103" t="n">
+      <c r="E103" t="n">
         <v>32.29</v>
       </c>
-      <c r="E103" t="n">
+      <c r="F103" t="n">
         <v>36.63</v>
       </c>
-      <c r="F103" t="n">
+      <c r="G103" t="n">
         <v>937821</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n">
         <v>42979</v>
       </c>
-      <c r="B104" t="n">
+      <c r="C104" t="n">
         <v>30.3</v>
       </c>
-      <c r="C104" t="n">
+      <c r="D104" t="n">
         <v>37</v>
       </c>
-      <c r="D104" t="n">
+      <c r="E104" t="n">
         <v>29.83</v>
       </c>
-      <c r="E104" t="n">
+      <c r="F104" t="n">
         <v>33.5</v>
       </c>
-      <c r="F104" t="n">
+      <c r="G104" t="n">
         <v>1266841</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="n">
         <v>42948</v>
       </c>
-      <c r="B105" t="n">
+      <c r="C105" t="n">
         <v>28.2</v>
       </c>
-      <c r="C105" t="n">
+      <c r="D105" t="n">
         <v>30.79</v>
       </c>
-      <c r="D105" t="n">
+      <c r="E105" t="n">
         <v>26.54</v>
       </c>
-      <c r="E105" t="n">
+      <c r="F105" t="n">
         <v>30.1</v>
       </c>
-      <c r="F105" t="n">
+      <c r="G105" t="n">
         <v>1119287</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="n">
         <v>42917</v>
       </c>
-      <c r="B106" t="n">
+      <c r="C106" t="n">
         <v>28.25</v>
       </c>
-      <c r="C106" t="n">
+      <c r="D106" t="n">
         <v>29.8</v>
       </c>
-      <c r="D106" t="n">
+      <c r="E106" t="n">
         <v>25.42</v>
       </c>
-      <c r="E106" t="n">
+      <c r="F106" t="n">
         <v>27.7</v>
       </c>
-      <c r="F106" t="n">
+      <c r="G106" t="n">
         <v>2236473</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>DHER.DE</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="n">
         <v>42887</v>
       </c>
-      <c r="B107" t="n">
+      <c r="C107" t="n">
         <v>26.9</v>
       </c>
-      <c r="C107" t="n">
+      <c r="D107" t="n">
         <v>27.8</v>
       </c>
-      <c r="D107" t="n">
+      <c r="E107" t="n">
         <v>25.26</v>
       </c>
-      <c r="E107" t="n">
+      <c r="F107" t="n">
         <v>27.8</v>
       </c>
-      <c r="F107" t="n">
+      <c r="G107" t="n">
         <v>11407039</v>
       </c>
     </row>

</xml_diff>